<commit_message>
Visualizzazione foto ad alta risoluzione con supporto PNG/JPEG/JPG
</commit_message>
<xml_diff>
--- a/data/catalogo.xlsx
+++ b/data/catalogo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF9366A3-786B-41EC-83B5-EBAD0C6E2ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEBA4E05-3500-4A6C-AE15-B1C4B51ACED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="160">
   <si>
     <t>ID</t>
   </si>
@@ -504,13 +504,28 @@
   </si>
   <si>
     <t>Organizzazioni_collegate</t>
+  </si>
+  <si>
+    <t>Nome_file</t>
+  </si>
+  <si>
+    <t>Delegazione PCd'I.jpg</t>
+  </si>
+  <si>
+    <t>1968.08.31, pag. 4 - Pesce e Mao.jpg</t>
+  </si>
+  <si>
+    <t>Renmin Ribao - 3 ottobre 1969, p.1 - Fosco Dinucci ai festeggiamenti RPC.jpg</t>
+  </si>
+  <si>
+    <t>Delegazione, ministero degli esteri.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -540,6 +555,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -562,18 +583,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -606,12 +642,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{27B22AD5-AC5E-42EE-98AF-49D8C6FF315D}" name="Tabella2" displayName="Tabella2" ref="A1:M32" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:M32" xr:uid="{27B22AD5-AC5E-42EE-98AF-49D8C6FF315D}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M31">
-    <sortCondition ref="A1:A31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{27B22AD5-AC5E-42EE-98AF-49D8C6FF315D}" name="Tabella2" displayName="Tabella2" ref="A1:N32" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:N32" xr:uid="{27B22AD5-AC5E-42EE-98AF-49D8C6FF315D}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N32">
+    <sortCondition ref="F1:F32"/>
   </sortState>
-  <tableColumns count="13">
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{2154B3EB-64E4-4E6D-8A0C-04D65D066E62}" name="ID"/>
     <tableColumn id="2" xr3:uid="{7C80280B-722C-4CED-A5F4-3F72F39F1DFC}" name="Titolo"/>
     <tableColumn id="3" xr3:uid="{42E23130-656A-4022-81E0-AF9117BAC245}" name="Organizzazione"/>
@@ -625,6 +661,7 @@
     <tableColumn id="9" xr3:uid="{18ED1BDE-DA2B-4274-908B-BC06AD7B6402}" name="Keywords"/>
     <tableColumn id="10" xr3:uid="{AEDEDEC1-9395-48B6-A4EF-01A581661641}" name="Note"/>
     <tableColumn id="11" xr3:uid="{575D6553-9BD2-40E4-8055-A706418FDCC7}" name="URL" dataCellStyle="Collegamento ipertestuale"/>
+    <tableColumn id="13" xr3:uid="{ACF3617F-A15C-4BA2-B462-292C6FA369C1}" name="Nome_file" dataDxfId="0" dataCellStyle="Collegamento ipertestuale"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -947,7 +984,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{342C46E2-AB3D-4CAD-AFB0-E7E2D6732CC9}">
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:O32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.21875" customWidth="1"/>
@@ -956,7 +993,7 @@
     <col min="11" max="11" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -996,16 +1033,20 @@
       <c r="M1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="O1" s="2"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
         <v>15</v>
@@ -1014,158 +1055,170 @@
         <v>1969</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
+        <v>80</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>84</v>
       </c>
       <c r="K2" t="s">
         <v>82</v>
       </c>
-      <c r="L2" t="s">
-        <v>13</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+      <c r="N2" s="5"/>
+      <c r="O2" s="2"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3">
-        <v>1967</v>
+        <v>57</v>
+      </c>
+      <c r="E3" s="3">
+        <v>25064</v>
       </c>
       <c r="F3" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G3" t="s">
         <v>11</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="K3" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+        <v>149</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="O3" s="2"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4">
-        <v>1968</v>
+        <v>60</v>
+      </c>
+      <c r="E4" s="3">
+        <v>25081</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G4" t="s">
         <v>11</v>
       </c>
       <c r="H4" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="K4" t="s">
-        <v>21</v>
+        <v>58</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="O4" s="2"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="B5" t="s">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5">
-        <v>1968</v>
+        <v>57</v>
+      </c>
+      <c r="E5" s="3">
+        <v>25479</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G5" t="s">
         <v>11</v>
       </c>
       <c r="H5" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="K5" t="s">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="O5" s="2"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>78</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6">
-        <v>1968</v>
+        <v>60</v>
+      </c>
+      <c r="E6" s="3">
+        <v>23511</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G6" t="s">
         <v>11</v>
       </c>
       <c r="H6" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="K6" t="s">
-        <v>26</v>
+        <v>71</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="O6" s="2"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -1174,10 +1227,10 @@
         <v>15</v>
       </c>
       <c r="E7">
-        <v>1968</v>
+        <v>1969</v>
       </c>
       <c r="F7" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
         <v>11</v>
@@ -1186,50 +1239,51 @@
         <v>18</v>
       </c>
       <c r="K7" t="s">
-        <v>30</v>
+        <v>82</v>
+      </c>
+      <c r="L7" t="s">
+        <v>13</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+        <v>140</v>
+      </c>
+      <c r="N7" s="5"/>
+      <c r="O7" s="2"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="D8" t="s">
-        <v>15</v>
+        <v>86</v>
       </c>
       <c r="E8">
-        <v>1968</v>
+        <v>1992</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H8" t="s">
-        <v>18</v>
+        <v>84</v>
       </c>
       <c r="K8" t="s">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+        <v>127</v>
+      </c>
+      <c r="N8" s="5"/>
+      <c r="O8" s="2"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
@@ -1238,7 +1292,7 @@
         <v>15</v>
       </c>
       <c r="E9">
-        <v>1969</v>
+        <v>1967</v>
       </c>
       <c r="F9" t="s">
         <v>20</v>
@@ -1250,18 +1304,20 @@
         <v>18</v>
       </c>
       <c r="K9" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+      <c r="N9" s="5"/>
+      <c r="O9" s="2"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1270,7 +1326,7 @@
         <v>15</v>
       </c>
       <c r="E10">
-        <v>1969</v>
+        <v>1968</v>
       </c>
       <c r="F10" t="s">
         <v>20</v>
@@ -1282,18 +1338,20 @@
         <v>18</v>
       </c>
       <c r="K10" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+        <v>138</v>
+      </c>
+      <c r="N10" s="5"/>
+      <c r="O10" s="2"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
@@ -1302,7 +1360,7 @@
         <v>15</v>
       </c>
       <c r="E11">
-        <v>1970</v>
+        <v>1968</v>
       </c>
       <c r="F11" t="s">
         <v>20</v>
@@ -1314,24 +1372,26 @@
         <v>18</v>
       </c>
       <c r="K11" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+        <v>137</v>
+      </c>
+      <c r="N11" s="5"/>
+      <c r="O11" s="2"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="E12">
         <v>1968</v>
@@ -1346,24 +1406,26 @@
         <v>18</v>
       </c>
       <c r="K12" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+      <c r="N12" s="5"/>
+      <c r="O12" s="2"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="E13">
         <v>1968</v>
@@ -1378,300 +1440,326 @@
         <v>18</v>
       </c>
       <c r="K13" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+        <v>136</v>
+      </c>
+      <c r="N13" s="5"/>
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>73</v>
+        <v>38</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="E14">
-        <v>1967</v>
+        <v>1968</v>
       </c>
       <c r="F14" t="s">
         <v>20</v>
       </c>
       <c r="G14" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="H14" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="K14" t="s">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+      <c r="N14" s="5"/>
+      <c r="O14" s="2"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>74</v>
+        <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
-      </c>
-      <c r="E15" s="3">
-        <v>25064</v>
+        <v>15</v>
+      </c>
+      <c r="E15">
+        <v>1969</v>
       </c>
       <c r="F15" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="G15" t="s">
         <v>11</v>
       </c>
       <c r="H15" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="K15" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+      <c r="N15" s="5"/>
+      <c r="O15" s="2"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D16" t="s">
-        <v>60</v>
-      </c>
-      <c r="E16" s="3">
-        <v>25081</v>
+        <v>15</v>
+      </c>
+      <c r="E16">
+        <v>1969</v>
       </c>
       <c r="F16" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="G16" t="s">
         <v>11</v>
       </c>
       <c r="H16" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="K16" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+      <c r="N16" s="5"/>
+      <c r="O16" s="2"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
-      </c>
-      <c r="E17" s="3">
-        <v>25479</v>
+        <v>15</v>
+      </c>
+      <c r="E17">
+        <v>1970</v>
       </c>
       <c r="F17" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="G17" t="s">
         <v>11</v>
       </c>
       <c r="H17" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="K17" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+      <c r="N17" s="5"/>
+      <c r="O17" s="2"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
-        <v>64</v>
+        <v>45</v>
       </c>
       <c r="C18" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>152</v>
-      </c>
-      <c r="E18" s="3">
-        <v>25485</v>
+        <v>46</v>
+      </c>
+      <c r="E18">
+        <v>1968</v>
       </c>
       <c r="F18" t="s">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="G18" t="s">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="H18" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="K18" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+      <c r="N18" s="5"/>
+      <c r="O18" s="2"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="C19" t="s">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="D19" t="s">
-        <v>60</v>
-      </c>
-      <c r="E19" s="3">
-        <v>23511</v>
+        <v>49</v>
+      </c>
+      <c r="E19">
+        <v>1968</v>
       </c>
       <c r="F19" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="G19" t="s">
         <v>11</v>
       </c>
       <c r="H19" t="s">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="K19" t="s">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+      <c r="N19" s="5"/>
+      <c r="O19" s="2"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>83</v>
+        <v>51</v>
       </c>
       <c r="D20" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20">
+        <v>1967</v>
+      </c>
+      <c r="F20" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" t="s">
+        <v>53</v>
+      </c>
+      <c r="H20" t="s">
+        <v>51</v>
+      </c>
+      <c r="K20" t="s">
+        <v>54</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="N20" s="5"/>
+      <c r="O20" s="2"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" t="s">
+        <v>97</v>
+      </c>
+      <c r="C21" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" t="s">
+        <v>98</v>
+      </c>
+      <c r="E21">
+        <v>1968</v>
+      </c>
+      <c r="F21" t="s">
+        <v>20</v>
+      </c>
+      <c r="G21" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" t="s">
+        <v>18</v>
+      </c>
+      <c r="K21" t="s">
+        <v>47</v>
+      </c>
+      <c r="M21" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="N21" s="5"/>
+      <c r="O21" s="2"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>147</v>
+      </c>
+      <c r="B22" t="s">
+        <v>145</v>
+      </c>
+      <c r="C22" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" t="s">
         <v>15</v>
       </c>
-      <c r="E20">
-        <v>1969</v>
-      </c>
-      <c r="F20" t="s">
-        <v>80</v>
-      </c>
-      <c r="H20" t="s">
-        <v>84</v>
-      </c>
-      <c r="K20" t="s">
-        <v>82</v>
-      </c>
-      <c r="M20" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>100</v>
-      </c>
-      <c r="B21" t="s">
-        <v>85</v>
-      </c>
-      <c r="D21" t="s">
-        <v>86</v>
-      </c>
-      <c r="E21">
-        <v>1992</v>
-      </c>
-      <c r="F21" t="s">
-        <v>10</v>
-      </c>
-      <c r="H21" t="s">
-        <v>84</v>
-      </c>
-      <c r="K21" t="s">
-        <v>87</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="E22">
+        <v>1968</v>
+      </c>
+      <c r="F22" t="s">
+        <v>20</v>
+      </c>
+      <c r="G22" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" t="s">
+        <v>18</v>
+      </c>
+      <c r="K22" t="s">
+        <v>146</v>
+      </c>
+      <c r="M22" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="N22" s="5"/>
+      <c r="O22" s="2"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
         <v>101</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>88</v>
-      </c>
-      <c r="C22" t="s">
-        <v>141</v>
-      </c>
-      <c r="D22" t="s">
-        <v>141</v>
-      </c>
-      <c r="E22" s="4">
-        <v>24746</v>
-      </c>
-      <c r="F22" t="s">
-        <v>151</v>
-      </c>
-      <c r="G22" t="s">
-        <v>142</v>
-      </c>
-      <c r="H22" t="s">
-        <v>114</v>
-      </c>
-      <c r="K22" t="s">
-        <v>113</v>
-      </c>
-      <c r="L22" t="s">
-        <v>144</v>
-      </c>
-      <c r="M22" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>102</v>
-      </c>
-      <c r="B23" t="s">
-        <v>89</v>
       </c>
       <c r="C23" t="s">
         <v>141</v>
@@ -1680,7 +1768,7 @@
         <v>141</v>
       </c>
       <c r="E23" s="4">
-        <v>24777</v>
+        <v>24746</v>
       </c>
       <c r="F23" t="s">
         <v>151</v>
@@ -1698,15 +1786,17 @@
         <v>144</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+        <v>126</v>
+      </c>
+      <c r="N23" s="5"/>
+      <c r="O23" s="2"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C24" t="s">
         <v>141</v>
@@ -1715,7 +1805,7 @@
         <v>141</v>
       </c>
       <c r="E24" s="4">
-        <v>24838</v>
+        <v>24777</v>
       </c>
       <c r="F24" t="s">
         <v>151</v>
@@ -1733,15 +1823,17 @@
         <v>144</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+      <c r="N24" s="5"/>
+      <c r="O24" s="2"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
         <v>141</v>
@@ -1750,7 +1842,7 @@
         <v>141</v>
       </c>
       <c r="E25" s="4">
-        <v>24869</v>
+        <v>24838</v>
       </c>
       <c r="F25" t="s">
         <v>151</v>
@@ -1768,15 +1860,17 @@
         <v>144</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+      <c r="N25" s="5"/>
+      <c r="O25" s="2"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B26" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C26" t="s">
         <v>141</v>
@@ -1785,7 +1879,7 @@
         <v>141</v>
       </c>
       <c r="E26" s="4">
-        <v>24898</v>
+        <v>24869</v>
       </c>
       <c r="F26" t="s">
         <v>151</v>
@@ -1803,15 +1897,17 @@
         <v>144</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+      <c r="N26" s="5"/>
+      <c r="O26" s="2"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B27" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C27" t="s">
         <v>141</v>
@@ -1820,7 +1916,7 @@
         <v>141</v>
       </c>
       <c r="E27" s="4">
-        <v>24959</v>
+        <v>24898</v>
       </c>
       <c r="F27" t="s">
         <v>151</v>
@@ -1829,24 +1925,26 @@
         <v>142</v>
       </c>
       <c r="H27" t="s">
-        <v>143</v>
+        <v>114</v>
       </c>
       <c r="K27" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L27" t="s">
         <v>144</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+      <c r="N27" s="5"/>
+      <c r="O27" s="2"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B28" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C28" t="s">
         <v>141</v>
@@ -1855,7 +1953,7 @@
         <v>141</v>
       </c>
       <c r="E28" s="4">
-        <v>24990</v>
+        <v>24959</v>
       </c>
       <c r="F28" t="s">
         <v>151</v>
@@ -1873,15 +1971,17 @@
         <v>144</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+      <c r="N28" s="5"/>
+      <c r="O28" s="2"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B29" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C29" t="s">
         <v>141</v>
@@ -1890,7 +1990,7 @@
         <v>141</v>
       </c>
       <c r="E29" s="4">
-        <v>25082</v>
+        <v>24990</v>
       </c>
       <c r="F29" t="s">
         <v>151</v>
@@ -1899,7 +1999,7 @@
         <v>142</v>
       </c>
       <c r="H29" t="s">
-        <v>116</v>
+        <v>143</v>
       </c>
       <c r="K29" t="s">
         <v>112</v>
@@ -1908,15 +2008,17 @@
         <v>144</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+        <v>119</v>
+      </c>
+      <c r="N29" s="5"/>
+      <c r="O29" s="2"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B30" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C30" t="s">
         <v>141</v>
@@ -1925,7 +2027,7 @@
         <v>141</v>
       </c>
       <c r="E30" s="4">
-        <v>25173</v>
+        <v>25082</v>
       </c>
       <c r="F30" t="s">
         <v>151</v>
@@ -1934,117 +2036,128 @@
         <v>142</v>
       </c>
       <c r="H30" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K30" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="L30" t="s">
         <v>144</v>
       </c>
       <c r="M30" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="N30" s="5"/>
+      <c r="O30" s="2"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>109</v>
+      </c>
+      <c r="B31" t="s">
+        <v>96</v>
+      </c>
+      <c r="C31" t="s">
+        <v>141</v>
+      </c>
+      <c r="D31" t="s">
+        <v>141</v>
+      </c>
+      <c r="E31" s="4">
+        <v>25173</v>
+      </c>
+      <c r="F31" t="s">
+        <v>151</v>
+      </c>
+      <c r="G31" t="s">
+        <v>142</v>
+      </c>
+      <c r="H31" t="s">
+        <v>115</v>
+      </c>
+      <c r="K31" t="s">
+        <v>111</v>
+      </c>
+      <c r="L31" t="s">
+        <v>144</v>
+      </c>
+      <c r="M31" s="1" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>110</v>
-      </c>
-      <c r="B31" t="s">
-        <v>97</v>
-      </c>
-      <c r="C31" t="s">
-        <v>12</v>
-      </c>
-      <c r="D31" t="s">
-        <v>98</v>
-      </c>
-      <c r="E31">
-        <v>1968</v>
-      </c>
-      <c r="F31" t="s">
-        <v>20</v>
-      </c>
-      <c r="G31" t="s">
-        <v>11</v>
-      </c>
-      <c r="H31" t="s">
-        <v>18</v>
-      </c>
-      <c r="K31" t="s">
-        <v>47</v>
-      </c>
-      <c r="M31" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N31" s="5"/>
+      <c r="O31" s="2"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>147</v>
+        <v>77</v>
       </c>
       <c r="B32" t="s">
-        <v>145</v>
+        <v>64</v>
       </c>
       <c r="C32" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="D32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E32">
-        <v>1968</v>
+        <v>152</v>
+      </c>
+      <c r="E32" s="3">
+        <v>25485</v>
       </c>
       <c r="F32" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="G32" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="H32" t="s">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="K32" t="s">
-        <v>146</v>
+        <v>68</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>148</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="N32" s="5"/>
+      <c r="O32" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="M2" r:id="rId1" xr:uid="{75651139-E161-458B-994F-5E49098574C4}"/>
-    <hyperlink ref="M3" r:id="rId2" xr:uid="{CD2184ED-A91F-4121-BCE4-6F5F57657BD3}"/>
-    <hyperlink ref="M5" r:id="rId3" xr:uid="{3151CD6F-6360-48A0-8A96-C6CA7BFA87B6}"/>
-    <hyperlink ref="M6" r:id="rId4" xr:uid="{921C0161-13F9-4AB1-9943-F088E8D04C77}"/>
-    <hyperlink ref="M7" r:id="rId5" xr:uid="{FA209DF6-7529-4AE3-93C8-C5B93022C678}"/>
-    <hyperlink ref="M8" r:id="rId6" xr:uid="{38D827A5-F723-490A-9D42-AA029CF987C7}"/>
-    <hyperlink ref="M9" r:id="rId7" xr:uid="{5EB7D969-3FFF-442C-88FB-72DAAAA56076}"/>
-    <hyperlink ref="M10" r:id="rId8" xr:uid="{2268931D-446D-439B-9355-E2623ED61D92}"/>
-    <hyperlink ref="M11" r:id="rId9" xr:uid="{915763FF-0C45-48F3-9200-2017B4DABB1A}"/>
-    <hyperlink ref="M4" r:id="rId10" xr:uid="{1F0EF04E-FA12-4EEF-97A1-C7749706DB4F}"/>
-    <hyperlink ref="M12" r:id="rId11" xr:uid="{EEE35428-6F4A-4888-8DC3-236CD045A4C4}"/>
-    <hyperlink ref="M13" r:id="rId12" xr:uid="{CD26B191-DAB6-4841-BD26-BA331F3F2FD5}"/>
-    <hyperlink ref="M16" r:id="rId13" xr:uid="{611B58DF-00D2-4FCD-BFD9-E1CB142D4AEA}"/>
-    <hyperlink ref="M18" r:id="rId14" xr:uid="{E315CB92-B7FC-4525-A8A4-456D931C2BB8}"/>
-    <hyperlink ref="M20" r:id="rId15" xr:uid="{3F906912-676F-47CF-9E8F-84EE32703C48}"/>
-    <hyperlink ref="M27" r:id="rId16" xr:uid="{7831D5F3-4CB5-4DC2-85FF-55351DC060AF}"/>
-    <hyperlink ref="M23" r:id="rId17" xr:uid="{C44BCAC6-AD3C-4236-BA13-54D5B6646DBA}"/>
-    <hyperlink ref="M30" r:id="rId18" xr:uid="{1C36EE42-0FF0-41A2-839A-2670099D91D7}"/>
-    <hyperlink ref="M28" r:id="rId19" xr:uid="{4715435A-D915-48BB-86DC-7EC994B95D73}"/>
-    <hyperlink ref="M29" r:id="rId20" xr:uid="{2406BBFC-AD68-471A-A754-E12E8DE9162D}"/>
-    <hyperlink ref="M31" r:id="rId21" xr:uid="{D78D0483-589F-4A18-B9C0-398C7F732239}"/>
-    <hyperlink ref="M24" r:id="rId22" xr:uid="{10936D2F-E6BF-4F7D-A904-6C00D4AC1D80}"/>
-    <hyperlink ref="M22" r:id="rId23" xr:uid="{96A5CD88-6692-4767-A93B-E739158B6BAB}"/>
-    <hyperlink ref="M21" r:id="rId24" xr:uid="{19EDCFD9-D88E-4993-A4E8-9BBF5848488C}"/>
-    <hyperlink ref="M14" r:id="rId25" xr:uid="{4D1018A8-1C5E-49D0-97C9-8DB65D890705}"/>
-    <hyperlink ref="M25" r:id="rId26" xr:uid="{68852D62-7997-4DA4-B0D6-64A7F310DAA6}"/>
-    <hyperlink ref="M32" r:id="rId27" xr:uid="{D4F6FC2F-CB40-4FC7-8086-063D674E2E9A}"/>
-    <hyperlink ref="M15" r:id="rId28" xr:uid="{7245A84A-A98E-4172-84DF-6CB6DA1C660D}"/>
+    <hyperlink ref="M7" r:id="rId1" xr:uid="{75651139-E161-458B-994F-5E49098574C4}"/>
+    <hyperlink ref="M9" r:id="rId2" xr:uid="{CD2184ED-A91F-4121-BCE4-6F5F57657BD3}"/>
+    <hyperlink ref="M11" r:id="rId3" xr:uid="{3151CD6F-6360-48A0-8A96-C6CA7BFA87B6}"/>
+    <hyperlink ref="M12" r:id="rId4" xr:uid="{921C0161-13F9-4AB1-9943-F088E8D04C77}"/>
+    <hyperlink ref="M13" r:id="rId5" xr:uid="{FA209DF6-7529-4AE3-93C8-C5B93022C678}"/>
+    <hyperlink ref="M14" r:id="rId6" xr:uid="{38D827A5-F723-490A-9D42-AA029CF987C7}"/>
+    <hyperlink ref="M15" r:id="rId7" xr:uid="{5EB7D969-3FFF-442C-88FB-72DAAAA56076}"/>
+    <hyperlink ref="M16" r:id="rId8" xr:uid="{2268931D-446D-439B-9355-E2623ED61D92}"/>
+    <hyperlink ref="M17" r:id="rId9" xr:uid="{915763FF-0C45-48F3-9200-2017B4DABB1A}"/>
+    <hyperlink ref="M10" r:id="rId10" xr:uid="{1F0EF04E-FA12-4EEF-97A1-C7749706DB4F}"/>
+    <hyperlink ref="M18" r:id="rId11" xr:uid="{EEE35428-6F4A-4888-8DC3-236CD045A4C4}"/>
+    <hyperlink ref="M19" r:id="rId12" xr:uid="{CD26B191-DAB6-4841-BD26-BA331F3F2FD5}"/>
+    <hyperlink ref="M4" r:id="rId13" xr:uid="{611B58DF-00D2-4FCD-BFD9-E1CB142D4AEA}"/>
+    <hyperlink ref="M32" r:id="rId14" xr:uid="{E315CB92-B7FC-4525-A8A4-456D931C2BB8}"/>
+    <hyperlink ref="M2" r:id="rId15" xr:uid="{3F906912-676F-47CF-9E8F-84EE32703C48}"/>
+    <hyperlink ref="M28" r:id="rId16" xr:uid="{7831D5F3-4CB5-4DC2-85FF-55351DC060AF}"/>
+    <hyperlink ref="M24" r:id="rId17" xr:uid="{C44BCAC6-AD3C-4236-BA13-54D5B6646DBA}"/>
+    <hyperlink ref="M31" r:id="rId18" xr:uid="{1C36EE42-0FF0-41A2-839A-2670099D91D7}"/>
+    <hyperlink ref="M29" r:id="rId19" xr:uid="{4715435A-D915-48BB-86DC-7EC994B95D73}"/>
+    <hyperlink ref="M30" r:id="rId20" xr:uid="{2406BBFC-AD68-471A-A754-E12E8DE9162D}"/>
+    <hyperlink ref="M21" r:id="rId21" xr:uid="{D78D0483-589F-4A18-B9C0-398C7F732239}"/>
+    <hyperlink ref="M25" r:id="rId22" xr:uid="{10936D2F-E6BF-4F7D-A904-6C00D4AC1D80}"/>
+    <hyperlink ref="M23" r:id="rId23" xr:uid="{96A5CD88-6692-4767-A93B-E739158B6BAB}"/>
+    <hyperlink ref="M8" r:id="rId24" xr:uid="{19EDCFD9-D88E-4993-A4E8-9BBF5848488C}"/>
+    <hyperlink ref="M20" r:id="rId25" xr:uid="{4D1018A8-1C5E-49D0-97C9-8DB65D890705}"/>
+    <hyperlink ref="M26" r:id="rId26" xr:uid="{68852D62-7997-4DA4-B0D6-64A7F310DAA6}"/>
+    <hyperlink ref="M22" r:id="rId27" xr:uid="{D4F6FC2F-CB40-4FC7-8086-063D674E2E9A}"/>
+    <hyperlink ref="M3" r:id="rId28" xr:uid="{7245A84A-A98E-4172-84DF-6CB6DA1C660D}"/>
+    <hyperlink ref="M5" r:id="rId29" xr:uid="{A1444548-667F-44FF-A262-FB159B81D88D}"/>
+    <hyperlink ref="M6" r:id="rId30" xr:uid="{EAA76073-A10F-44D7-BE5A-B85456ABE721}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId29"/>
+    <tablePart r:id="rId31"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Supporto visualizzazione file .txt da Internet Archive
</commit_message>
<xml_diff>
--- a/data/catalogo.xlsx
+++ b/data/catalogo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEBA4E05-3500-4A6C-AE15-B1C4B51ACED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7772B68-2A7C-4323-8C1D-07563A6E2C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="168">
   <si>
     <t>ID</t>
   </si>
@@ -519,6 +519,30 @@
   </si>
   <si>
     <t>Delegazione, ministero degli esteri.jpg</t>
+  </si>
+  <si>
+    <t>Statuto di Stella Rossa - Fronte Rivoluzionario Marxista-Leninista</t>
+  </si>
+  <si>
+    <t>Stella Rossa - Fronte Rivoluzionario Marxista-Leninista</t>
+  </si>
+  <si>
+    <t>AMI-0032</t>
+  </si>
+  <si>
+    <t>Testo</t>
+  </si>
+  <si>
+    <t>Galassia m-l</t>
+  </si>
+  <si>
+    <t>Vincenzo Calò</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/statuto-stella-rossa</t>
+  </si>
+  <si>
+    <t>STATUTO DI STELLA ROSSA.txt</t>
   </si>
 </sst>
 </file>
@@ -642,10 +666,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{27B22AD5-AC5E-42EE-98AF-49D8C6FF315D}" name="Tabella2" displayName="Tabella2" ref="A1:N32" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:N32" xr:uid="{27B22AD5-AC5E-42EE-98AF-49D8C6FF315D}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N32">
-    <sortCondition ref="F1:F32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{27B22AD5-AC5E-42EE-98AF-49D8C6FF315D}" name="Tabella2" displayName="Tabella2" ref="A1:N51" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:N51" xr:uid="{27B22AD5-AC5E-42EE-98AF-49D8C6FF315D}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N51">
+    <sortCondition ref="A1:A51"/>
   </sortState>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{2154B3EB-64E4-4E6D-8A0C-04D65D066E62}" name="ID"/>
@@ -984,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{342C46E2-AB3D-4CAD-AFB0-E7E2D6732CC9}">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.21875" customWidth="1"/>
@@ -1040,13 +1064,13 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>99</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
         <v>15</v>
@@ -1055,170 +1079,168 @@
         <v>1969</v>
       </c>
       <c r="F2" t="s">
-        <v>80</v>
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
       </c>
       <c r="H2" t="s">
-        <v>84</v>
+        <v>18</v>
       </c>
       <c r="K2" t="s">
         <v>82</v>
       </c>
+      <c r="L2" t="s">
+        <v>13</v>
+      </c>
       <c r="M2" s="1" t="s">
-        <v>81</v>
+        <v>140</v>
       </c>
       <c r="N2" s="5"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E3" s="3">
-        <v>25064</v>
+        <v>15</v>
+      </c>
+      <c r="E3">
+        <v>1967</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="G3" t="s">
         <v>11</v>
       </c>
       <c r="H3" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="K3" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>156</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="N3" s="5"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E4" s="3">
-        <v>25081</v>
+        <v>15</v>
+      </c>
+      <c r="E4">
+        <v>1968</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="G4" t="s">
         <v>11</v>
       </c>
       <c r="H4" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="K4" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N4" s="5" t="s">
-        <v>157</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="N4" s="5"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E5" s="3">
-        <v>25479</v>
+        <v>15</v>
+      </c>
+      <c r="E5">
+        <v>1968</v>
       </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="G5" t="s">
         <v>11</v>
       </c>
       <c r="H5" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="K5" t="s">
-        <v>58</v>
+        <v>24</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>158</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="N5" s="5"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E6" s="3">
-        <v>23511</v>
+        <v>15</v>
+      </c>
+      <c r="E6">
+        <v>1968</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="G6" t="s">
         <v>11</v>
       </c>
       <c r="H6" t="s">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="K6" t="s">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>159</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="N6" s="5"/>
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
         <v>12</v>
@@ -1227,10 +1249,10 @@
         <v>15</v>
       </c>
       <c r="E7">
-        <v>1969</v>
+        <v>1968</v>
       </c>
       <c r="F7" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="G7" t="s">
         <v>11</v>
@@ -1239,51 +1261,54 @@
         <v>18</v>
       </c>
       <c r="K7" t="s">
-        <v>82</v>
-      </c>
-      <c r="L7" t="s">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="N7" s="5"/>
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>100</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>86</v>
+        <v>15</v>
       </c>
       <c r="E8">
-        <v>1992</v>
+        <v>1968</v>
       </c>
       <c r="F8" t="s">
-        <v>10</v>
+        <v>20</v>
+      </c>
+      <c r="G8" t="s">
+        <v>11</v>
       </c>
       <c r="H8" t="s">
-        <v>84</v>
+        <v>18</v>
       </c>
       <c r="K8" t="s">
-        <v>87</v>
+        <v>30</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="N8" s="5"/>
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
@@ -1292,7 +1317,7 @@
         <v>15</v>
       </c>
       <c r="E9">
-        <v>1967</v>
+        <v>1969</v>
       </c>
       <c r="F9" t="s">
         <v>20</v>
@@ -1304,20 +1329,20 @@
         <v>18</v>
       </c>
       <c r="K9" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="N9" s="5"/>
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1326,7 +1351,7 @@
         <v>15</v>
       </c>
       <c r="E10">
-        <v>1968</v>
+        <v>1969</v>
       </c>
       <c r="F10" t="s">
         <v>20</v>
@@ -1338,20 +1363,20 @@
         <v>18</v>
       </c>
       <c r="K10" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="N10" s="5"/>
       <c r="O10" s="2"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
@@ -1360,7 +1385,7 @@
         <v>15</v>
       </c>
       <c r="E11">
-        <v>1968</v>
+        <v>1970</v>
       </c>
       <c r="F11" t="s">
         <v>20</v>
@@ -1372,26 +1397,26 @@
         <v>18</v>
       </c>
       <c r="K11" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="N11" s="5"/>
       <c r="O11" s="2"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="E12">
         <v>1968</v>
@@ -1406,26 +1431,26 @@
         <v>18</v>
       </c>
       <c r="K12" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>27</v>
+        <v>131</v>
       </c>
       <c r="N12" s="5"/>
       <c r="O12" s="2"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="E13">
         <v>1968</v>
@@ -1440,326 +1465,328 @@
         <v>18</v>
       </c>
       <c r="K13" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="N13" s="5"/>
       <c r="O13" s="2"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>50</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D14" t="s">
-        <v>15</v>
+        <v>52</v>
       </c>
       <c r="E14">
-        <v>1968</v>
+        <v>1967</v>
       </c>
       <c r="F14" t="s">
         <v>20</v>
       </c>
       <c r="G14" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="H14" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="K14" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="N14" s="5"/>
       <c r="O14" s="2"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D15" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15">
-        <v>1969</v>
+        <v>57</v>
+      </c>
+      <c r="E15" s="3">
+        <v>25064</v>
       </c>
       <c r="F15" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G15" t="s">
         <v>11</v>
       </c>
       <c r="H15" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="K15" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="N15" s="5"/>
+        <v>149</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>156</v>
+      </c>
       <c r="O15" s="2"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16">
-        <v>1969</v>
+        <v>60</v>
+      </c>
+      <c r="E16" s="3">
+        <v>25081</v>
       </c>
       <c r="F16" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G16" t="s">
         <v>11</v>
       </c>
       <c r="H16" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="K16" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="N16" s="5"/>
+        <v>61</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>157</v>
+      </c>
       <c r="O16" s="2"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="D17" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17">
-        <v>1970</v>
+        <v>57</v>
+      </c>
+      <c r="E17" s="3">
+        <v>25479</v>
       </c>
       <c r="F17" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G17" t="s">
         <v>11</v>
       </c>
       <c r="H17" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="K17" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="N17" s="5"/>
+        <v>63</v>
+      </c>
+      <c r="N17" s="5" t="s">
+        <v>158</v>
+      </c>
       <c r="O17" s="2"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>77</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="C18" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="D18" t="s">
-        <v>46</v>
-      </c>
-      <c r="E18">
-        <v>1968</v>
+        <v>152</v>
+      </c>
+      <c r="E18" s="3">
+        <v>25485</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="G18" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="H18" t="s">
-        <v>18</v>
+        <v>67</v>
       </c>
       <c r="K18" t="s">
-        <v>47</v>
+        <v>68</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="N18" s="5"/>
       <c r="O18" s="2"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
-        <v>48</v>
+        <v>69</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="D19" t="s">
-        <v>49</v>
-      </c>
-      <c r="E19">
-        <v>1968</v>
+        <v>60</v>
+      </c>
+      <c r="E19" s="3">
+        <v>23511</v>
       </c>
       <c r="F19" t="s">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G19" t="s">
         <v>11</v>
       </c>
       <c r="H19" t="s">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="K19" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="N19" s="5"/>
+        <v>72</v>
+      </c>
+      <c r="N19" s="5" t="s">
+        <v>159</v>
+      </c>
       <c r="O19" s="2"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>73</v>
+        <v>99</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>83</v>
       </c>
       <c r="D20" t="s">
-        <v>52</v>
+        <v>15</v>
       </c>
       <c r="E20">
-        <v>1967</v>
+        <v>1969</v>
       </c>
       <c r="F20" t="s">
-        <v>20</v>
-      </c>
-      <c r="G20" t="s">
-        <v>53</v>
+        <v>80</v>
       </c>
       <c r="H20" t="s">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="K20" t="s">
-        <v>54</v>
+        <v>82</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>129</v>
+        <v>81</v>
       </c>
       <c r="N20" s="5"/>
       <c r="O20" s="2"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B21" t="s">
-        <v>97</v>
-      </c>
-      <c r="C21" t="s">
-        <v>12</v>
+        <v>85</v>
       </c>
       <c r="D21" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="E21">
-        <v>1968</v>
+        <v>1992</v>
       </c>
       <c r="F21" t="s">
-        <v>20</v>
-      </c>
-      <c r="G21" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H21" t="s">
-        <v>18</v>
+        <v>84</v>
       </c>
       <c r="K21" t="s">
-        <v>47</v>
+        <v>87</v>
       </c>
       <c r="M21" s="1" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="N21" s="5"/>
       <c r="O21" s="2"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>147</v>
+        <v>101</v>
       </c>
       <c r="B22" t="s">
-        <v>145</v>
+        <v>88</v>
       </c>
       <c r="C22" t="s">
-        <v>12</v>
+        <v>141</v>
       </c>
       <c r="D22" t="s">
-        <v>15</v>
-      </c>
-      <c r="E22">
-        <v>1968</v>
+        <v>141</v>
+      </c>
+      <c r="E22" s="4">
+        <v>24746</v>
       </c>
       <c r="F22" t="s">
-        <v>20</v>
+        <v>151</v>
       </c>
       <c r="G22" t="s">
-        <v>11</v>
+        <v>142</v>
       </c>
       <c r="H22" t="s">
-        <v>18</v>
+        <v>114</v>
       </c>
       <c r="K22" t="s">
-        <v>146</v>
+        <v>113</v>
+      </c>
+      <c r="L22" t="s">
+        <v>144</v>
       </c>
       <c r="M22" s="1" t="s">
-        <v>148</v>
+        <v>126</v>
       </c>
       <c r="N22" s="5"/>
       <c r="O22" s="2"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C23" t="s">
         <v>141</v>
@@ -1768,7 +1795,7 @@
         <v>141</v>
       </c>
       <c r="E23" s="4">
-        <v>24746</v>
+        <v>24777</v>
       </c>
       <c r="F23" t="s">
         <v>151</v>
@@ -1786,17 +1813,17 @@
         <v>144</v>
       </c>
       <c r="M23" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N23" s="5"/>
       <c r="O23" s="2"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B24" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
         <v>141</v>
@@ -1805,7 +1832,7 @@
         <v>141</v>
       </c>
       <c r="E24" s="4">
-        <v>24777</v>
+        <v>24838</v>
       </c>
       <c r="F24" t="s">
         <v>151</v>
@@ -1823,17 +1850,17 @@
         <v>144</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="N24" s="5"/>
       <c r="O24" s="2"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
         <v>141</v>
@@ -1842,7 +1869,7 @@
         <v>141</v>
       </c>
       <c r="E25" s="4">
-        <v>24838</v>
+        <v>24869</v>
       </c>
       <c r="F25" t="s">
         <v>151</v>
@@ -1860,17 +1887,17 @@
         <v>144</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="N25" s="5"/>
       <c r="O25" s="2"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B26" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C26" t="s">
         <v>141</v>
@@ -1879,7 +1906,7 @@
         <v>141</v>
       </c>
       <c r="E26" s="4">
-        <v>24869</v>
+        <v>24898</v>
       </c>
       <c r="F26" t="s">
         <v>151</v>
@@ -1897,17 +1924,17 @@
         <v>144</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="N26" s="5"/>
       <c r="O26" s="2"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C27" t="s">
         <v>141</v>
@@ -1916,7 +1943,7 @@
         <v>141</v>
       </c>
       <c r="E27" s="4">
-        <v>24898</v>
+        <v>24959</v>
       </c>
       <c r="F27" t="s">
         <v>151</v>
@@ -1925,26 +1952,26 @@
         <v>142</v>
       </c>
       <c r="H27" t="s">
-        <v>114</v>
+        <v>143</v>
       </c>
       <c r="K27" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L27" t="s">
         <v>144</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="N27" s="5"/>
       <c r="O27" s="2"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B28" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C28" t="s">
         <v>141</v>
@@ -1953,7 +1980,7 @@
         <v>141</v>
       </c>
       <c r="E28" s="4">
-        <v>24959</v>
+        <v>24990</v>
       </c>
       <c r="F28" t="s">
         <v>151</v>
@@ -1971,17 +1998,17 @@
         <v>144</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="N28" s="5"/>
       <c r="O28" s="2"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B29" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C29" t="s">
         <v>141</v>
@@ -1990,7 +2017,7 @@
         <v>141</v>
       </c>
       <c r="E29" s="4">
-        <v>24990</v>
+        <v>25082</v>
       </c>
       <c r="F29" t="s">
         <v>151</v>
@@ -1999,7 +2026,7 @@
         <v>142</v>
       </c>
       <c r="H29" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="K29" t="s">
         <v>112</v>
@@ -2008,17 +2035,17 @@
         <v>144</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="N29" s="5"/>
       <c r="O29" s="2"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C30" t="s">
         <v>141</v>
@@ -2027,7 +2054,7 @@
         <v>141</v>
       </c>
       <c r="E30" s="4">
-        <v>25082</v>
+        <v>25173</v>
       </c>
       <c r="F30" t="s">
         <v>151</v>
@@ -2036,124 +2063,228 @@
         <v>142</v>
       </c>
       <c r="H30" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K30" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L30" t="s">
         <v>144</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N30" s="5"/>
       <c r="O30" s="2"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B31" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C31" t="s">
-        <v>141</v>
+        <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>141</v>
-      </c>
-      <c r="E31" s="4">
-        <v>25173</v>
+        <v>98</v>
+      </c>
+      <c r="E31">
+        <v>1968</v>
       </c>
       <c r="F31" t="s">
-        <v>151</v>
+        <v>20</v>
       </c>
       <c r="G31" t="s">
-        <v>142</v>
+        <v>11</v>
       </c>
       <c r="H31" t="s">
-        <v>115</v>
+        <v>18</v>
       </c>
       <c r="K31" t="s">
-        <v>111</v>
-      </c>
-      <c r="L31" t="s">
-        <v>144</v>
+        <v>47</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N31" s="5"/>
       <c r="O31" s="2"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>77</v>
+        <v>147</v>
       </c>
       <c r="B32" t="s">
-        <v>64</v>
+        <v>145</v>
       </c>
       <c r="C32" t="s">
-        <v>65</v>
+        <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>152</v>
-      </c>
-      <c r="E32" s="3">
-        <v>25485</v>
+        <v>15</v>
+      </c>
+      <c r="E32">
+        <v>1968</v>
       </c>
       <c r="F32" t="s">
-        <v>150</v>
+        <v>20</v>
       </c>
       <c r="G32" t="s">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="H32" t="s">
-        <v>67</v>
+        <v>18</v>
       </c>
       <c r="K32" t="s">
-        <v>68</v>
+        <v>146</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
       <c r="N32" s="5"/>
       <c r="O32" s="2"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>162</v>
+      </c>
+      <c r="B33" t="s">
+        <v>160</v>
+      </c>
+      <c r="C33" t="s">
+        <v>161</v>
+      </c>
+      <c r="D33" t="s">
+        <v>161</v>
+      </c>
+      <c r="E33">
+        <v>1970</v>
+      </c>
+      <c r="F33" t="s">
+        <v>163</v>
+      </c>
+      <c r="H33" t="s">
+        <v>164</v>
+      </c>
+      <c r="I33" t="s">
+        <v>165</v>
+      </c>
+      <c r="K33" t="s">
+        <v>113</v>
+      </c>
+      <c r="M33" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="N33" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M34" s="1"/>
+      <c r="N34" s="5"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M35" s="1"/>
+      <c r="N35" s="5"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M36" s="1"/>
+      <c r="N36" s="5"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M37" s="1"/>
+      <c r="N37" s="5"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M38" s="1"/>
+      <c r="N38" s="5"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M39" s="1"/>
+      <c r="N39" s="5"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M40" s="1"/>
+      <c r="N40" s="5"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M41" s="1"/>
+      <c r="N41" s="5"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M42" s="1"/>
+      <c r="N42" s="5"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M43" s="1"/>
+      <c r="N43" s="5"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M44" s="1"/>
+      <c r="N44" s="5"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M45" s="1"/>
+      <c r="N45" s="5"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M46" s="1"/>
+      <c r="N46" s="5"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M47" s="1"/>
+      <c r="N47" s="5"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M48" s="1"/>
+      <c r="N48" s="5"/>
+    </row>
+    <row r="49" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M49" s="1"/>
+      <c r="N49" s="5"/>
+    </row>
+    <row r="50" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M50" s="1"/>
+      <c r="N50" s="5"/>
+    </row>
+    <row r="51" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M51" s="1"/>
+      <c r="N51" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="M7" r:id="rId1" xr:uid="{75651139-E161-458B-994F-5E49098574C4}"/>
-    <hyperlink ref="M9" r:id="rId2" xr:uid="{CD2184ED-A91F-4121-BCE4-6F5F57657BD3}"/>
-    <hyperlink ref="M11" r:id="rId3" xr:uid="{3151CD6F-6360-48A0-8A96-C6CA7BFA87B6}"/>
-    <hyperlink ref="M12" r:id="rId4" xr:uid="{921C0161-13F9-4AB1-9943-F088E8D04C77}"/>
-    <hyperlink ref="M13" r:id="rId5" xr:uid="{FA209DF6-7529-4AE3-93C8-C5B93022C678}"/>
-    <hyperlink ref="M14" r:id="rId6" xr:uid="{38D827A5-F723-490A-9D42-AA029CF987C7}"/>
-    <hyperlink ref="M15" r:id="rId7" xr:uid="{5EB7D969-3FFF-442C-88FB-72DAAAA56076}"/>
-    <hyperlink ref="M16" r:id="rId8" xr:uid="{2268931D-446D-439B-9355-E2623ED61D92}"/>
-    <hyperlink ref="M17" r:id="rId9" xr:uid="{915763FF-0C45-48F3-9200-2017B4DABB1A}"/>
-    <hyperlink ref="M10" r:id="rId10" xr:uid="{1F0EF04E-FA12-4EEF-97A1-C7749706DB4F}"/>
-    <hyperlink ref="M18" r:id="rId11" xr:uid="{EEE35428-6F4A-4888-8DC3-236CD045A4C4}"/>
-    <hyperlink ref="M19" r:id="rId12" xr:uid="{CD26B191-DAB6-4841-BD26-BA331F3F2FD5}"/>
-    <hyperlink ref="M4" r:id="rId13" xr:uid="{611B58DF-00D2-4FCD-BFD9-E1CB142D4AEA}"/>
-    <hyperlink ref="M32" r:id="rId14" xr:uid="{E315CB92-B7FC-4525-A8A4-456D931C2BB8}"/>
-    <hyperlink ref="M2" r:id="rId15" xr:uid="{3F906912-676F-47CF-9E8F-84EE32703C48}"/>
-    <hyperlink ref="M28" r:id="rId16" xr:uid="{7831D5F3-4CB5-4DC2-85FF-55351DC060AF}"/>
-    <hyperlink ref="M24" r:id="rId17" xr:uid="{C44BCAC6-AD3C-4236-BA13-54D5B6646DBA}"/>
-    <hyperlink ref="M31" r:id="rId18" xr:uid="{1C36EE42-0FF0-41A2-839A-2670099D91D7}"/>
-    <hyperlink ref="M29" r:id="rId19" xr:uid="{4715435A-D915-48BB-86DC-7EC994B95D73}"/>
-    <hyperlink ref="M30" r:id="rId20" xr:uid="{2406BBFC-AD68-471A-A754-E12E8DE9162D}"/>
-    <hyperlink ref="M21" r:id="rId21" xr:uid="{D78D0483-589F-4A18-B9C0-398C7F732239}"/>
-    <hyperlink ref="M25" r:id="rId22" xr:uid="{10936D2F-E6BF-4F7D-A904-6C00D4AC1D80}"/>
-    <hyperlink ref="M23" r:id="rId23" xr:uid="{96A5CD88-6692-4767-A93B-E739158B6BAB}"/>
-    <hyperlink ref="M8" r:id="rId24" xr:uid="{19EDCFD9-D88E-4993-A4E8-9BBF5848488C}"/>
-    <hyperlink ref="M20" r:id="rId25" xr:uid="{4D1018A8-1C5E-49D0-97C9-8DB65D890705}"/>
-    <hyperlink ref="M26" r:id="rId26" xr:uid="{68852D62-7997-4DA4-B0D6-64A7F310DAA6}"/>
-    <hyperlink ref="M22" r:id="rId27" xr:uid="{D4F6FC2F-CB40-4FC7-8086-063D674E2E9A}"/>
-    <hyperlink ref="M3" r:id="rId28" xr:uid="{7245A84A-A98E-4172-84DF-6CB6DA1C660D}"/>
-    <hyperlink ref="M5" r:id="rId29" xr:uid="{A1444548-667F-44FF-A262-FB159B81D88D}"/>
-    <hyperlink ref="M6" r:id="rId30" xr:uid="{EAA76073-A10F-44D7-BE5A-B85456ABE721}"/>
+    <hyperlink ref="M2" r:id="rId1" xr:uid="{75651139-E161-458B-994F-5E49098574C4}"/>
+    <hyperlink ref="M3" r:id="rId2" xr:uid="{CD2184ED-A91F-4121-BCE4-6F5F57657BD3}"/>
+    <hyperlink ref="M5" r:id="rId3" xr:uid="{3151CD6F-6360-48A0-8A96-C6CA7BFA87B6}"/>
+    <hyperlink ref="M6" r:id="rId4" xr:uid="{921C0161-13F9-4AB1-9943-F088E8D04C77}"/>
+    <hyperlink ref="M7" r:id="rId5" xr:uid="{FA209DF6-7529-4AE3-93C8-C5B93022C678}"/>
+    <hyperlink ref="M8" r:id="rId6" xr:uid="{38D827A5-F723-490A-9D42-AA029CF987C7}"/>
+    <hyperlink ref="M9" r:id="rId7" xr:uid="{5EB7D969-3FFF-442C-88FB-72DAAAA56076}"/>
+    <hyperlink ref="M10" r:id="rId8" xr:uid="{2268931D-446D-439B-9355-E2623ED61D92}"/>
+    <hyperlink ref="M11" r:id="rId9" xr:uid="{915763FF-0C45-48F3-9200-2017B4DABB1A}"/>
+    <hyperlink ref="M4" r:id="rId10" xr:uid="{1F0EF04E-FA12-4EEF-97A1-C7749706DB4F}"/>
+    <hyperlink ref="M12" r:id="rId11" xr:uid="{EEE35428-6F4A-4888-8DC3-236CD045A4C4}"/>
+    <hyperlink ref="M13" r:id="rId12" xr:uid="{CD26B191-DAB6-4841-BD26-BA331F3F2FD5}"/>
+    <hyperlink ref="M16" r:id="rId13" xr:uid="{611B58DF-00D2-4FCD-BFD9-E1CB142D4AEA}"/>
+    <hyperlink ref="M18" r:id="rId14" xr:uid="{E315CB92-B7FC-4525-A8A4-456D931C2BB8}"/>
+    <hyperlink ref="M20" r:id="rId15" xr:uid="{3F906912-676F-47CF-9E8F-84EE32703C48}"/>
+    <hyperlink ref="M27" r:id="rId16" xr:uid="{7831D5F3-4CB5-4DC2-85FF-55351DC060AF}"/>
+    <hyperlink ref="M23" r:id="rId17" xr:uid="{C44BCAC6-AD3C-4236-BA13-54D5B6646DBA}"/>
+    <hyperlink ref="M30" r:id="rId18" xr:uid="{1C36EE42-0FF0-41A2-839A-2670099D91D7}"/>
+    <hyperlink ref="M28" r:id="rId19" xr:uid="{4715435A-D915-48BB-86DC-7EC994B95D73}"/>
+    <hyperlink ref="M29" r:id="rId20" xr:uid="{2406BBFC-AD68-471A-A754-E12E8DE9162D}"/>
+    <hyperlink ref="M31" r:id="rId21" xr:uid="{D78D0483-589F-4A18-B9C0-398C7F732239}"/>
+    <hyperlink ref="M24" r:id="rId22" xr:uid="{10936D2F-E6BF-4F7D-A904-6C00D4AC1D80}"/>
+    <hyperlink ref="M22" r:id="rId23" xr:uid="{96A5CD88-6692-4767-A93B-E739158B6BAB}"/>
+    <hyperlink ref="M21" r:id="rId24" xr:uid="{19EDCFD9-D88E-4993-A4E8-9BBF5848488C}"/>
+    <hyperlink ref="M14" r:id="rId25" xr:uid="{4D1018A8-1C5E-49D0-97C9-8DB65D890705}"/>
+    <hyperlink ref="M25" r:id="rId26" xr:uid="{68852D62-7997-4DA4-B0D6-64A7F310DAA6}"/>
+    <hyperlink ref="M32" r:id="rId27" xr:uid="{D4F6FC2F-CB40-4FC7-8086-063D674E2E9A}"/>
+    <hyperlink ref="M15" r:id="rId28" xr:uid="{7245A84A-A98E-4172-84DF-6CB6DA1C660D}"/>
+    <hyperlink ref="M17" r:id="rId29" xr:uid="{A1444548-667F-44FF-A262-FB159B81D88D}"/>
+    <hyperlink ref="M19" r:id="rId30" xr:uid="{EAA76073-A10F-44D7-BE5A-B85456ABE721}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 02/08/2026 09:11
</commit_message>
<xml_diff>
--- a/data/catalogo.xlsx
+++ b/data/catalogo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{215150F6-4860-4BB6-BF41-55F4F3B4897C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36CEDE61-1C4A-4FFA-B421-47742D9ADF6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3864" yWindow="1596" windowWidth="17280" windowHeight="8880" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="259">
   <si>
     <t>ID</t>
   </si>
@@ -780,6 +780,42 @@
   </si>
   <si>
     <t>Sosteniamo il Congresso di fondazione del PARTITO COMUNISTA (marxista-leninista) ITALIANO per fare l'Italia rossa e socialista come la Cina di Mao</t>
+  </si>
+  <si>
+    <t>AMI-0054</t>
+  </si>
+  <si>
+    <t>AMI-0055</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/manifesto-pcudi-breznev</t>
+  </si>
+  <si>
+    <t>manifesto-pcudi-breznev.jpg</t>
+  </si>
+  <si>
+    <t>Osvaldo Pesce</t>
+  </si>
+  <si>
+    <t>Manifesto</t>
+  </si>
+  <si>
+    <t>Linea Proletaria</t>
+  </si>
+  <si>
+    <t>Partito Comunista Unificato d'Italia</t>
+  </si>
+  <si>
+    <t>RICERCATO: Leonida Breznev - Manifesto del Partito Comunista Unificato d'Italia</t>
+  </si>
+  <si>
+    <t>Osare pensare, osare parlare, osare agire, osare fare la rivoluzione - Manifesto PCd'I (m-l)</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/osare-poster-pcdi</t>
+  </si>
+  <si>
+    <t>osare-poster-pcdi.png</t>
   </si>
 </sst>
 </file>
@@ -3080,12 +3116,74 @@
       <c r="M54" s="5"/>
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="L55" s="1"/>
-      <c r="M55" s="5"/>
+      <c r="A55" t="s">
+        <v>247</v>
+      </c>
+      <c r="B55" t="s">
+        <v>255</v>
+      </c>
+      <c r="C55" t="s">
+        <v>254</v>
+      </c>
+      <c r="D55" t="s">
+        <v>254</v>
+      </c>
+      <c r="E55" t="s">
+        <v>253</v>
+      </c>
+      <c r="F55">
+        <v>1978</v>
+      </c>
+      <c r="G55" t="s">
+        <v>252</v>
+      </c>
+      <c r="H55" t="s">
+        <v>161</v>
+      </c>
+      <c r="I55" t="s">
+        <v>165</v>
+      </c>
+      <c r="J55" t="s">
+        <v>251</v>
+      </c>
+      <c r="L55" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="M55" s="5" t="s">
+        <v>250</v>
+      </c>
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="L56" s="1"/>
-      <c r="M56" s="5"/>
+      <c r="A56" t="s">
+        <v>248</v>
+      </c>
+      <c r="B56" t="s">
+        <v>256</v>
+      </c>
+      <c r="C56" t="s">
+        <v>41</v>
+      </c>
+      <c r="D56" t="s">
+        <v>41</v>
+      </c>
+      <c r="E56" t="s">
+        <v>48</v>
+      </c>
+      <c r="F56">
+        <v>1967</v>
+      </c>
+      <c r="G56" t="s">
+        <v>252</v>
+      </c>
+      <c r="I56" t="s">
+        <v>165</v>
+      </c>
+      <c r="L56" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="M56" s="5" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="L57" s="1"/>

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 02/08/2026 12:34
</commit_message>
<xml_diff>
--- a/data/catalogo.xlsx
+++ b/data/catalogo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36CEDE61-1C4A-4FFA-B421-47742D9ADF6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42E4B5E3-6365-47ED-B909-C36574E3EA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="267">
   <si>
     <t>ID</t>
   </si>
@@ -816,6 +816,30 @@
   </si>
   <si>
     <t>osare-poster-pcdi.png</t>
+  </si>
+  <si>
+    <t>AMI-0056</t>
+  </si>
+  <si>
+    <t>Il Presidente Mao Tse-tung sulla Guerra di popolo</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/mao-tse-tung-guerra-di-popolo/mode/2up</t>
+  </si>
+  <si>
+    <t>AMI-0057</t>
+  </si>
+  <si>
+    <t>Congresso di fondazione del Partito Comunista d'Italia</t>
+  </si>
+  <si>
+    <t>https://archive.org/details/fondazione-pcudi-1977</t>
+  </si>
+  <si>
+    <t>fondazione-pcudi-1977.jpg</t>
+  </si>
+  <si>
+    <t>Organizzazione dei Comunisti (marxisti-leninisti) d'Italia; Organizzazione Comunista (marxista-leninista) - Fronte Unito; Partito Comunista d'Italia (marxista-leninista) - Lotta di lunga; Partito Marxista-Leninista-Maoista Italiano</t>
   </si>
 </sst>
 </file>
@@ -1289,7 +1313,7 @@
     <col min="2" max="2" width="53.5546875" customWidth="1"/>
     <col min="3" max="4" width="20.77734375" customWidth="1"/>
     <col min="5" max="5" width="12.77734375" customWidth="1"/>
-    <col min="6" max="6" width="10.77734375" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" customWidth="1"/>
     <col min="8" max="8" width="22.5546875" customWidth="1"/>
     <col min="9" max="9" width="11.109375" customWidth="1"/>
     <col min="10" max="10" width="22.44140625" customWidth="1"/>
@@ -3131,8 +3155,8 @@
       <c r="E55" t="s">
         <v>253</v>
       </c>
-      <c r="F55">
-        <v>1978</v>
+      <c r="F55" s="4">
+        <v>28550</v>
       </c>
       <c r="G55" t="s">
         <v>252</v>
@@ -3186,12 +3210,78 @@
       </c>
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="L57" s="1"/>
+      <c r="A57" t="s">
+        <v>259</v>
+      </c>
+      <c r="B57" t="s">
+        <v>260</v>
+      </c>
+      <c r="C57" t="s">
+        <v>56</v>
+      </c>
+      <c r="D57" t="s">
+        <v>13</v>
+      </c>
+      <c r="E57" t="s">
+        <v>56</v>
+      </c>
+      <c r="F57">
+        <v>1967</v>
+      </c>
+      <c r="G57" t="s">
+        <v>9</v>
+      </c>
+      <c r="H57" t="s">
+        <v>161</v>
+      </c>
+      <c r="I57" t="s">
+        <v>196</v>
+      </c>
+      <c r="L57" s="1" t="s">
+        <v>261</v>
+      </c>
       <c r="M57" s="5"/>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="L58" s="1"/>
-      <c r="M58" s="5"/>
+      <c r="A58" t="s">
+        <v>262</v>
+      </c>
+      <c r="B58" t="s">
+        <v>263</v>
+      </c>
+      <c r="C58" t="s">
+        <v>254</v>
+      </c>
+      <c r="D58" t="s">
+        <v>254</v>
+      </c>
+      <c r="E58" t="s">
+        <v>253</v>
+      </c>
+      <c r="F58" s="3">
+        <v>28253</v>
+      </c>
+      <c r="G58" t="s">
+        <v>44</v>
+      </c>
+      <c r="H58" t="s">
+        <v>169</v>
+      </c>
+      <c r="I58" t="s">
+        <v>165</v>
+      </c>
+      <c r="J58" t="s">
+        <v>251</v>
+      </c>
+      <c r="K58" t="s">
+        <v>266</v>
+      </c>
+      <c r="L58" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="M58" s="5" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="L59" s="1"/>
@@ -3542,11 +3632,12 @@
     <hyperlink ref="L52" r:id="rId48" xr:uid="{6D6C9EBD-C509-45AC-AD32-2A67AD2727AD}"/>
     <hyperlink ref="L53" r:id="rId49" xr:uid="{A01892A1-954B-41E4-B4CB-95523808FE8E}"/>
     <hyperlink ref="L54" r:id="rId50" xr:uid="{5A52ABF7-103B-48A3-9933-A864844B57D6}"/>
+    <hyperlink ref="L57" r:id="rId51" xr:uid="{09F4A066-8FFE-45CF-800B-1E59F7E2C7C3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId51"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId52"/>
   <tableParts count="1">
-    <tablePart r:id="rId52"/>
+    <tablePart r:id="rId53"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 02/08/2026 14:14
</commit_message>
<xml_diff>
--- a/data/catalogo.xlsx
+++ b/data/catalogo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42E4B5E3-6365-47ED-B909-C36574E3EA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9889F5D0-D2C1-4524-9904-27A56E52E1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
+    <workbookView xWindow="348" yWindow="3060" windowWidth="17280" windowHeight="8880" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -836,10 +836,10 @@
     <t>https://archive.org/details/fondazione-pcudi-1977</t>
   </si>
   <si>
-    <t>fondazione-pcudi-1977.jpg</t>
-  </si>
-  <si>
     <t>Organizzazione dei Comunisti (marxisti-leninisti) d'Italia; Organizzazione Comunista (marxista-leninista) - Fronte Unito; Partito Comunista d'Italia (marxista-leninista) - Lotta di lunga; Partito Marxista-Leninista-Maoista Italiano</t>
+  </si>
+  <si>
+    <t>05.08.1977-fondazione-pcudi.png</t>
   </si>
 </sst>
 </file>
@@ -3274,13 +3274,13 @@
         <v>251</v>
       </c>
       <c r="K58" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="L58" s="1" t="s">
         <v>264</v>
       </c>
       <c r="M58" s="5" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Aggiornamento automatico del sito — 02/08/2026 21:16
</commit_message>
<xml_diff>
--- a/data/catalogo.xlsx
+++ b/data/catalogo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ivan_\Desktop\AMI\GitHub\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9889F5D0-D2C1-4524-9904-27A56E52E1F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB79B241-F61F-4688-8816-F9A4B511AF06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="348" yWindow="3060" windowWidth="17280" windowHeight="8880" xr2:uid="{F5AF1365-4D1F-4A73-8F23-4ABAB32F4B91}"/>
   </bookViews>
@@ -830,9 +830,6 @@
     <t>AMI-0057</t>
   </si>
   <si>
-    <t>Congresso di fondazione del Partito Comunista d'Italia</t>
-  </si>
-  <si>
     <t>https://archive.org/details/fondazione-pcudi-1977</t>
   </si>
   <si>
@@ -840,6 +837,9 @@
   </si>
   <si>
     <t>05.08.1977-fondazione-pcudi.png</t>
+  </si>
+  <si>
+    <t>Congresso di fondazione del Partito Comunista Unificato d'Italia</t>
   </si>
 </sst>
 </file>
@@ -3247,7 +3247,7 @@
         <v>262</v>
       </c>
       <c r="B58" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C58" t="s">
         <v>254</v>
@@ -3274,13 +3274,13 @@
         <v>251</v>
       </c>
       <c r="K58" t="s">
+        <v>264</v>
+      </c>
+      <c r="L58" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="M58" s="5" t="s">
         <v>265</v>
-      </c>
-      <c r="L58" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="M58" s="5" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>